<commit_message>
CMGJ-7 Actualizado Excel de requisitos
</commit_message>
<xml_diff>
--- a/definition/Generated/Requirements.xlsx
+++ b/definition/Generated/Requirements.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cgomezji\TFM\definition\Generated\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlos\Documents\MSEI\TFM\definition\Generated\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0DA8B1C3-0C08-4944-BA64-665054362CCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2BAD973-5783-4B83-BE9C-4456411433EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requisitos" sheetId="1" r:id="rId1"/>
+    <sheet name="Listas" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
@@ -191,7 +192,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="42">
   <si>
     <t>Id</t>
   </si>
@@ -214,12 +215,6 @@
     <t>R1.1</t>
   </si>
   <si>
-    <t>Temperatura</t>
-  </si>
-  <si>
-    <t>El sistema medirá la temperatura de todas las máquinas.</t>
-  </si>
-  <si>
     <t>F</t>
   </si>
   <si>
@@ -229,212 +224,107 @@
     <t>R1.2</t>
   </si>
   <si>
-    <t>Velocidad</t>
-  </si>
-  <si>
-    <t>El sistema medirá la velocidad de las máquinas con rollo.</t>
-  </si>
-  <si>
-    <t>R1.3</t>
-  </si>
-  <si>
-    <t>Presión</t>
-  </si>
-  <si>
-    <t>El sistema medirá la presión de aire de las máquinas extrusoras.</t>
-  </si>
-  <si>
     <t>R2.1</t>
   </si>
   <si>
-    <t>MostrarTemperatura</t>
-  </si>
-  <si>
-    <t>El sistema mostrará la temperatura en el PC de la oficina.</t>
-  </si>
-  <si>
     <t>R2.2</t>
   </si>
   <si>
-    <t>MostrarVelocidad</t>
-  </si>
-  <si>
-    <t>El sistema mostrará la velocidad en el PC de la oficina.</t>
-  </si>
-  <si>
     <t>R2.3</t>
   </si>
   <si>
-    <t>MostrarPresión</t>
-  </si>
-  <si>
-    <t>El sistema mostrará la presión en el PC de la oficina.</t>
-  </si>
-  <si>
     <t>R2.4</t>
   </si>
   <si>
-    <t>MostrarAlarmas</t>
-  </si>
-  <si>
-    <t>El sistema mostrará las alarmas en el PC de la oficina.</t>
-  </si>
-  <si>
-    <t>R1.1,R11</t>
-  </si>
-  <si>
-    <t>R3</t>
-  </si>
-  <si>
-    <t>ActuarRefrige</t>
-  </si>
-  <si>
-    <t>El sistema permitirá parar las máquinas en las que se mide la temperatura.</t>
-  </si>
-  <si>
     <t>D</t>
   </si>
   <si>
-    <t>R4</t>
-  </si>
-  <si>
-    <t>RestriccionActuarRefrige</t>
-  </si>
-  <si>
-    <t>Sólo se pararán las máquinas con temperatura fuera de rango.</t>
-  </si>
-  <si>
-    <t>R1.1, R3</t>
-  </si>
-  <si>
-    <t>No Funcional</t>
-  </si>
-  <si>
-    <t>R5</t>
-  </si>
-  <si>
     <t>FechaEntrega</t>
   </si>
   <si>
-    <t>El proyecto debe finalizar el 18/12/2014 (1 mes y medio después de la primera reunión)</t>
-  </si>
-  <si>
-    <t>R6.1</t>
-  </si>
-  <si>
-    <t>AñadirMaquinasTemperatura</t>
-  </si>
-  <si>
-    <t>El sistema debe permitir añadir más maquinas para medir Temperatura una vez entregado</t>
-  </si>
-  <si>
-    <t>R1.1, R2.1</t>
-  </si>
-  <si>
-    <t>R6.2</t>
-  </si>
-  <si>
-    <t>AñadirMaquinasVelocidad</t>
-  </si>
-  <si>
-    <t>El sistema debe permitir añadir más maquinas para medir Velocidad una vez entregado</t>
-  </si>
-  <si>
-    <t>R1.2, R2.2</t>
-  </si>
-  <si>
-    <t>R6.3</t>
-  </si>
-  <si>
-    <t>AñadirMaquinasPresión</t>
-  </si>
-  <si>
-    <t>El sistema debe permitir añadir más maquinas para medir Presión una vez entregado</t>
-  </si>
-  <si>
-    <t>R1.3, R2.3</t>
-  </si>
-  <si>
-    <t>R7</t>
-  </si>
-  <si>
-    <t>ValorTempatura</t>
-  </si>
-  <si>
-    <t>El sistema debe permitir medir temperaturas de hasta 400 ºC</t>
-  </si>
-  <si>
-    <t>R1.1, R2</t>
-  </si>
-  <si>
-    <t>R8</t>
-  </si>
-  <si>
-    <t>GuardarHistorico</t>
-  </si>
-  <si>
-    <t>El sistema almacenará todas las lecturas y las alarmas en un histórico en el PC de la oficina del cliente</t>
-  </si>
-  <si>
-    <t>R1.*</t>
-  </si>
-  <si>
-    <t>R9</t>
-  </si>
-  <si>
-    <t>MaximoHistorico</t>
-  </si>
-  <si>
-    <t>El sistema almacenará el histórico durante 1 año.</t>
-  </si>
-  <si>
-    <t>R10.1</t>
-  </si>
-  <si>
-    <t>ActualizaciónDatos</t>
-  </si>
-  <si>
-    <t>Los datos se leen cada 5 minutos.</t>
-  </si>
-  <si>
-    <t>R1.* R2.*</t>
-  </si>
-  <si>
-    <t>R10.2</t>
-  </si>
-  <si>
-    <t>AlmacenajeDatos</t>
-  </si>
-  <si>
-    <t>Los datos se almacenan cada 5 minutos.</t>
-  </si>
-  <si>
-    <t>R1.* R2.*, R8</t>
-  </si>
-  <si>
-    <t>R11</t>
-  </si>
-  <si>
-    <t>RangoAlarma</t>
-  </si>
-  <si>
-    <t>Los valores válidos de temperatura se almacenarán en un fichero de texto plano según la máquina.</t>
-  </si>
-  <si>
-    <t>R12</t>
-  </si>
-  <si>
-    <t>Ganancias</t>
-  </si>
-  <si>
-    <t>Las ganancias deben ser de 3000 euros (2000 por mes)</t>
+    <t>Prioridades</t>
+  </si>
+  <si>
+    <t>O</t>
+  </si>
+  <si>
+    <t>No funcional</t>
+  </si>
+  <si>
+    <t>La fecha de entrega Final será el XX/XX/XX</t>
+  </si>
+  <si>
+    <t>FechaHito</t>
+  </si>
+  <si>
+    <t>Habrá un hito previo a la entrega Final para demostrar el correcto funcionamiento del proyecto hasta el XX/XX/XX</t>
+  </si>
+  <si>
+    <t>SensorCamara</t>
+  </si>
+  <si>
+    <t>ConexionSensor</t>
+  </si>
+  <si>
+    <t>ConexionHost</t>
+  </si>
+  <si>
+    <t>HostCamara</t>
+  </si>
+  <si>
+    <t>El sensor de imagen (cámara) utilizado es el modelo MT9V111. Referencia XX en Lista de Materiales (LM)</t>
+  </si>
+  <si>
+    <t>La conexión del sensor con el host se realizará de forma directa: pin a pin con el adaptador proporcionado. Referencia XX en Lista de Materiales (LM)</t>
+  </si>
+  <si>
+    <t>El Host encargado de comunicar el sensor con el ordenador es la FPGA Basys3. Referencia XX en Lista de Materiales (LM)</t>
+  </si>
+  <si>
+    <t>La conexión del host con el ordenador se realiza mediante un cable USB-microUSB (TBC)</t>
+  </si>
+  <si>
+    <t>FrecuenciaImagen</t>
+  </si>
+  <si>
+    <t>La Frecuencia mínima a la que deben llegar las imágenes por la comunicación serie al PC es de TBC Hz</t>
+  </si>
+  <si>
+    <t>El sensor debe configurarse para capturar una resolución mínima de XxX</t>
+  </si>
+  <si>
+    <t>El retardo total desde la captura del frame hasta su visualización en el PC no debe superar los X ms</t>
+  </si>
+  <si>
+    <t>El software en el PC debe mostrar el flujo de vídeo en una ventana dedicada</t>
+  </si>
+  <si>
+    <t>ResolucionMinima</t>
+  </si>
+  <si>
+    <t>RetardoMaximo</t>
+  </si>
+  <si>
+    <t>VentanaGUI</t>
+  </si>
+  <si>
+    <t>R2.5</t>
+  </si>
+  <si>
+    <t>R2.6</t>
+  </si>
+  <si>
+    <t>R2.7</t>
+  </si>
+  <si>
+    <t>R2.8</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -470,6 +360,19 @@
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -479,7 +382,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -502,13 +405,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="hair">
+        <color auto="1"/>
+      </left>
+      <right style="hair">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1147,7 +1063,7 @@
   <cols>
     <col min="1" max="1" width="8"/>
     <col min="2" max="2" width="24.5703125"/>
-    <col min="3" max="3" width="88"/>
+    <col min="3" max="3" width="129.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.5703125"/>
     <col min="5" max="5" width="15.5703125"/>
     <col min="6" max="6" width="13.5703125"/>
@@ -1186,407 +1102,263 @@
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G2" s="1"/>
     </row>
     <row r="3" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G3" s="1"/>
     </row>
     <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G4" s="1"/>
     </row>
     <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>18</v>
+        <v>11</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>23</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>6</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="E5" s="1"/>
       <c r="F5" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G5" s="1"/>
     </row>
     <row r="6" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>11</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="E6" s="1"/>
       <c r="F6" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G6" s="1"/>
     </row>
     <row r="7" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>14</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="E7" s="1"/>
       <c r="F7" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G7" s="1"/>
     </row>
     <row r="8" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>10</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
       <c r="G8" s="1"/>
     </row>
     <row r="9" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>10</v>
-      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
       <c r="G9" s="1"/>
     </row>
     <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="C10" t="s">
         <v>33</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>38</v>
-      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
       <c r="G10" s="1"/>
     </row>
     <row r="11" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>9</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="C11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" s="1"/>
       <c r="E11" s="1"/>
-      <c r="F11" s="1" t="s">
-        <v>38</v>
-      </c>
+      <c r="F11" s="1"/>
       <c r="G11" s="1"/>
     </row>
     <row r="12" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>10</v>
-      </c>
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
       <c r="G12" s="1"/>
     </row>
     <row r="13" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>10</v>
-      </c>
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
       <c r="G13" s="1"/>
     </row>
     <row r="14" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>10</v>
-      </c>
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
       <c r="G14" s="1"/>
     </row>
     <row r="15" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>38</v>
-      </c>
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
       <c r="G15" s="1"/>
     </row>
     <row r="16" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>10</v>
-      </c>
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
       <c r="G16" s="1"/>
     </row>
     <row r="17" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>38</v>
-      </c>
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
       <c r="G17" s="1"/>
     </row>
     <row r="18" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>38</v>
-      </c>
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
       <c r="G18" s="1"/>
     </row>
     <row r="19" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>38</v>
-      </c>
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
       <c r="G19" s="1"/>
     </row>
     <row r="20" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>33</v>
-      </c>
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
       <c r="E20" s="1"/>
-      <c r="F20" s="1" t="s">
-        <v>10</v>
-      </c>
+      <c r="F20" s="1"/>
       <c r="G20" s="1"/>
     </row>
     <row r="21" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>33</v>
-      </c>
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
       <c r="E21" s="1"/>
-      <c r="F21" s="1" t="s">
-        <v>38</v>
-      </c>
+      <c r="F21" s="1"/>
       <c r="G21" s="1"/>
     </row>
     <row r="22" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1599,10 +1371,73 @@
       <c r="G22" s="1"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="6" type="noConversion"/>
+  <dataValidations disablePrompts="1" count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E7" xr:uid="{4DDBC533-0419-46F1-B6B3-324F26BF199B}">
+      <formula1>$A$2:$A$1048576</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="0" scale="0" firstPageNumber="0" orientation="portrait" usePrinterDefaults="0" horizontalDpi="0" verticalDpi="0" copies="0"/>
   <drawing r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="2">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B376F8AC-A9ED-42D4-87E9-8777062C6B21}">
+          <x14:formula1>
+            <xm:f>Listas!$A$2:$A$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>D2:D7</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{93332DCB-95CB-47BB-B0B8-5373262B883D}">
+          <x14:formula1>
+            <xm:f>Listas!$B$2:$B$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>F2:F7</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A245119-F5B4-4F14-8676-0240AA483E11}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
CMGJ-7 #time 30m nuevo proyecto con sysml 14 y modificacion de requisitos
</commit_message>
<xml_diff>
--- a/definition/Generated/Requirements.xlsx
+++ b/definition/Generated/Requirements.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlos\Documents\MSEI\TFM\definition\Generated\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2BAD973-5783-4B83-BE9C-4456411433EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CE23AF6-E21D-4BB2-91CE-3B802A391DB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requisitos" sheetId="1" r:id="rId1"/>
     <sheet name="Listas" sheetId="2" r:id="rId2"/>
+    <sheet name="LM" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
@@ -56,7 +57,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -82,7 +83,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
       <text>
         <r>
           <rPr>
@@ -108,7 +109,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
       <text>
         <r>
           <rPr>
@@ -137,7 +138,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
+    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
       <text>
         <r>
           <rPr>
@@ -163,7 +164,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
       <text>
         <r>
           <rPr>
@@ -192,10 +193,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="42">
-  <si>
-    <t>Id</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="59">
   <si>
     <t>Nombre</t>
   </si>
@@ -212,36 +210,15 @@
     <t>Tipo</t>
   </si>
   <si>
-    <t>R1.1</t>
-  </si>
-  <si>
     <t>F</t>
   </si>
   <si>
     <t>Funcional</t>
   </si>
   <si>
-    <t>R1.2</t>
-  </si>
-  <si>
-    <t>R2.1</t>
-  </si>
-  <si>
-    <t>R2.2</t>
-  </si>
-  <si>
-    <t>R2.3</t>
-  </si>
-  <si>
-    <t>R2.4</t>
-  </si>
-  <si>
     <t>D</t>
   </si>
   <si>
-    <t>FechaEntrega</t>
-  </si>
-  <si>
     <t>Prioridades</t>
   </si>
   <si>
@@ -251,15 +228,6 @@
     <t>No funcional</t>
   </si>
   <si>
-    <t>La fecha de entrega Final será el XX/XX/XX</t>
-  </si>
-  <si>
-    <t>FechaHito</t>
-  </si>
-  <si>
-    <t>Habrá un hito previo a la entrega Final para demostrar el correcto funcionamiento del proyecto hasta el XX/XX/XX</t>
-  </si>
-  <si>
     <t>SensorCamara</t>
   </si>
   <si>
@@ -287,9 +255,6 @@
     <t>FrecuenciaImagen</t>
   </si>
   <si>
-    <t>La Frecuencia mínima a la que deben llegar las imágenes por la comunicación serie al PC es de TBC Hz</t>
-  </si>
-  <si>
     <t>El sensor debe configurarse para capturar una resolución mínima de XxX</t>
   </si>
   <si>
@@ -308,16 +273,103 @@
     <t>VentanaGUI</t>
   </si>
   <si>
-    <t>R2.5</t>
-  </si>
-  <si>
-    <t>R2.6</t>
-  </si>
-  <si>
-    <t>R2.7</t>
-  </si>
-  <si>
-    <t>R2.8</t>
+    <t>FechaEntregaOrd</t>
+  </si>
+  <si>
+    <t>FechaEntregaExt</t>
+  </si>
+  <si>
+    <t>FechaHito (TBC)</t>
+  </si>
+  <si>
+    <t>Habrá un hito previo a la entrega Final para demostrar el correcto funcionamiento del proyecto hasta el TBD</t>
+  </si>
+  <si>
+    <t>La Frecuencia mínima a la que deben llegar las imágenes por la comunicación serie al PC es de TBD Hz</t>
+  </si>
+  <si>
+    <t>La fecha de entrega Final será el TBD para la convocatoria Extraordinaria</t>
+  </si>
+  <si>
+    <t>La fecha de entrega Final será el TBD para la convocatoria Ordinaria</t>
+  </si>
+  <si>
+    <t>Referencia</t>
+  </si>
+  <si>
+    <t>SPN</t>
+  </si>
+  <si>
+    <t>MPN</t>
+  </si>
+  <si>
+    <t>Unidades</t>
+  </si>
+  <si>
+    <t>BASYS3</t>
+  </si>
+  <si>
+    <t>B1</t>
+  </si>
+  <si>
+    <t>B2</t>
+  </si>
+  <si>
+    <t>CAMARA CMOS</t>
+  </si>
+  <si>
+    <t>InterfazHostHS</t>
+  </si>
+  <si>
+    <t>La interfaz del Host con el PC se realizará con la tarjeta UM232H-B (TBC). Referencia XX en la Lista de Materiales (LM)</t>
+  </si>
+  <si>
+    <t>El lenguaje de programación utilizado para el desarrollo del software encargado del procesamiento de imagen será TBD</t>
+  </si>
+  <si>
+    <t>LenguajeOpenCV</t>
+  </si>
+  <si>
+    <t>Se permite y se insta al uso de librerías de procesamiento de imágenes como OpenCV</t>
+  </si>
+  <si>
+    <t>UsoOpenCV</t>
+  </si>
+  <si>
+    <t>La cámara será configurable a nivel TBD</t>
+  </si>
+  <si>
+    <t>Los parámetros de configuración de la cámara son: TBD</t>
+  </si>
+  <si>
+    <t>ConfiguracionCamara</t>
+  </si>
+  <si>
+    <t>ParametrosConfiguracion</t>
+  </si>
+  <si>
+    <t>BotonesGUI</t>
+  </si>
+  <si>
+    <t>La ventana dedicada permitirá el control/configuración de TBD</t>
+  </si>
+  <si>
+    <t>Id1</t>
+  </si>
+  <si>
+    <t>Id2</t>
+  </si>
+  <si>
+    <t>UM232H-B</t>
+  </si>
+  <si>
+    <t>Ordenador</t>
+  </si>
+  <si>
+    <t>El PC encargado de ejecutar el SW tiene el SO Windows (TBD) con las siguientes capacidades mínimas: TBD</t>
+  </si>
+  <si>
+    <t>Memoria</t>
   </si>
 </sst>
 </file>
@@ -420,16 +472,44 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -452,9 +532,9 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
+      <xdr:col>5</xdr:col>
       <xdr:colOff>781050</xdr:colOff>
-      <xdr:row>50</xdr:row>
+      <xdr:row>52</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -501,9 +581,9 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
+      <xdr:col>5</xdr:col>
       <xdr:colOff>781050</xdr:colOff>
-      <xdr:row>50</xdr:row>
+      <xdr:row>52</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -550,9 +630,9 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
+      <xdr:col>5</xdr:col>
       <xdr:colOff>781050</xdr:colOff>
-      <xdr:row>50</xdr:row>
+      <xdr:row>52</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -599,9 +679,9 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
+      <xdr:col>5</xdr:col>
       <xdr:colOff>781050</xdr:colOff>
-      <xdr:row>50</xdr:row>
+      <xdr:row>52</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -648,9 +728,9 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
+      <xdr:col>5</xdr:col>
       <xdr:colOff>781050</xdr:colOff>
-      <xdr:row>50</xdr:row>
+      <xdr:row>52</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -697,9 +777,9 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
+      <xdr:col>5</xdr:col>
       <xdr:colOff>781050</xdr:colOff>
-      <xdr:row>50</xdr:row>
+      <xdr:row>52</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -739,6 +819,21 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9B14786E-76C0-4757-8667-4880971DAF80}" name="Tabla1" displayName="Tabla1" ref="B2:G5" totalsRowShown="0">
+  <autoFilter ref="B2:G5" xr:uid="{9B14786E-76C0-4757-8667-4880971DAF80}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{A0410A85-38BB-4A45-AEE3-330768CE3424}" name="Referencia" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{D058449A-B7D8-4DC9-BDD0-571A11974A46}" name="MPN"/>
+    <tableColumn id="3" xr3:uid="{FFC1C329-DDE7-4CE2-A73E-13C0903E7F19}" name="SPN"/>
+    <tableColumn id="4" xr3:uid="{EC2A09CA-662B-46BF-AD5F-EBDAD89E9A5E}" name="Nombre"/>
+    <tableColumn id="5" xr3:uid="{ED9C3681-DD83-4CE3-8CEA-65D38A08E7B4}" name="Unidades" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{4E1825E6-4FDD-41A5-9263-0B196EA0C97F}" name="Descripción"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1058,16 +1153,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8"/>
-    <col min="2" max="2" width="24.5703125"/>
-    <col min="3" max="3" width="129.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5703125"/>
-    <col min="5" max="5" width="15.5703125"/>
-    <col min="6" max="6" width="13.5703125"/>
-    <col min="7" max="7" width="14.28515625"/>
+    <col min="3" max="3" width="24.5703125"/>
+    <col min="4" max="4" width="129.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" style="4"/>
+    <col min="6" max="6" width="15.5703125"/>
+    <col min="7" max="7" width="13.5703125"/>
     <col min="8" max="8" width="15.85546875"/>
     <col min="9" max="9" width="12.85546875"/>
     <col min="10" max="10" width="14.85546875"/>
@@ -1077,287 +1171,431 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1"/>
     </row>
     <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>1</v>
+      </c>
+      <c r="B4" s="1">
+        <v>3</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>2</v>
+      </c>
+      <c r="B5" s="1">
+        <v>1</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="1" t="s">
+    </row>
+    <row r="6" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>2</v>
+      </c>
+      <c r="B6" s="1">
+        <v>2</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>2</v>
+      </c>
+      <c r="B7" s="3">
+        <v>1</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>2</v>
+      </c>
+      <c r="B8" s="3">
+        <v>1</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>3</v>
+      </c>
+      <c r="B9" s="1">
+        <v>2</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>4</v>
+      </c>
+      <c r="B10" s="1">
+        <v>1</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>4</v>
+      </c>
+      <c r="B11" s="1">
+        <v>2</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>4</v>
+      </c>
+      <c r="B12" s="1">
+        <v>3</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>5</v>
+      </c>
+      <c r="B13" s="1">
+        <v>1</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="5">
+        <v>6</v>
+      </c>
+      <c r="B14" s="5">
+        <v>1</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" t="s">
+        <v>22</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="5">
+        <v>6</v>
+      </c>
+      <c r="B15" s="5">
+        <v>2</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D15" t="s">
+        <v>52</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
         <v>7</v>
       </c>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" s="1"/>
-    </row>
-    <row r="3" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="B16" s="1">
+        <v>1</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>7</v>
+      </c>
+      <c r="B17" s="1">
+        <v>2</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>8</v>
+      </c>
+      <c r="B18" s="1">
+        <v>1</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>8</v>
+      </c>
+      <c r="B19" s="1">
+        <v>2</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
         <v>9</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" s="1"/>
-    </row>
-    <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="B20" s="1">
+        <v>1</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="E20" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G4" s="1"/>
-    </row>
-    <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G5" s="1"/>
-    </row>
-    <row r="6" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G6" s="1"/>
-    </row>
-    <row r="7" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G7" s="1"/>
-    </row>
-    <row r="8" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-    </row>
-    <row r="9" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-    </row>
-    <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10" t="s">
-        <v>33</v>
-      </c>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-    </row>
-    <row r="11" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C11" t="s">
-        <v>34</v>
-      </c>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-    </row>
-    <row r="12" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-    </row>
-    <row r="13" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-    </row>
-    <row r="14" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-    </row>
-    <row r="15" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-    </row>
-    <row r="16" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-    </row>
-    <row r="17" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-    </row>
-    <row r="18" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-    </row>
-    <row r="19" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-    </row>
-    <row r="20" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
     </row>
     <row r="21" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
+      <c r="E21" s="6"/>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
     </row>
@@ -1366,14 +1604,40 @@
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
+      <c r="E22" s="6"/>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
     </row>
+    <row r="23" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+    </row>
+    <row r="24" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
+  <conditionalFormatting sqref="A1:XFD1048576">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="TBD">
+      <formula>NOT(ISERROR(SEARCH("TBD",A1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="TBC">
+      <formula>NOT(ISERROR(SEARCH("TBC",A1)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations disablePrompts="1" count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E7" xr:uid="{4DDBC533-0419-46F1-B6B3-324F26BF199B}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F20" xr:uid="{4DDBC533-0419-46F1-B6B3-324F26BF199B}">
       <formula1>$A$2:$A$1048576</formula1>
     </dataValidation>
   </dataValidations>
@@ -1388,13 +1652,13 @@
           <x14:formula1>
             <xm:f>Listas!$A$2:$A$4</xm:f>
           </x14:formula1>
-          <xm:sqref>D2:D7</xm:sqref>
+          <xm:sqref>E2:E20</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{93332DCB-95CB-47BB-B0B8-5373262B883D}">
           <x14:formula1>
             <xm:f>Listas!$B$2:$B$3</xm:f>
           </x14:formula1>
-          <xm:sqref>F2:F7</xm:sqref>
+          <xm:sqref>G2:G20</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1409,35 +1673,101 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E4E333C-009A-4DDD-A904-57A4DE1A7306}">
+  <dimension ref="B2:G5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="12.7109375" style="4" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" style="4" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B2" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B3" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B4" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="E5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
CMGJ-13 #time 2h Empezado con EF22, sin acabar todavía
</commit_message>
<xml_diff>
--- a/definition/Generated/Requirements.xlsx
+++ b/definition/Generated/Requirements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlos\Documents\MSEI\TFM\definition\Generated\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CE23AF6-E21D-4BB2-91CE-3B802A391DB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A0B3E0A-E379-4DCB-A732-28F70A6C977E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requisitos" sheetId="1" r:id="rId1"/>
@@ -193,7 +193,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="70">
   <si>
     <t>Nombre</t>
   </si>
@@ -249,21 +249,9 @@
     <t>El Host encargado de comunicar el sensor con el ordenador es la FPGA Basys3. Referencia XX en Lista de Materiales (LM)</t>
   </si>
   <si>
-    <t>La conexión del host con el ordenador se realiza mediante un cable USB-microUSB (TBC)</t>
-  </si>
-  <si>
     <t>FrecuenciaImagen</t>
   </si>
   <si>
-    <t>El sensor debe configurarse para capturar una resolución mínima de XxX</t>
-  </si>
-  <si>
-    <t>El retardo total desde la captura del frame hasta su visualización en el PC no debe superar los X ms</t>
-  </si>
-  <si>
-    <t>El software en el PC debe mostrar el flujo de vídeo en una ventana dedicada</t>
-  </si>
-  <si>
     <t>ResolucionMinima</t>
   </si>
   <si>
@@ -279,21 +267,6 @@
     <t>FechaEntregaExt</t>
   </si>
   <si>
-    <t>FechaHito (TBC)</t>
-  </si>
-  <si>
-    <t>Habrá un hito previo a la entrega Final para demostrar el correcto funcionamiento del proyecto hasta el TBD</t>
-  </si>
-  <si>
-    <t>La Frecuencia mínima a la que deben llegar las imágenes por la comunicación serie al PC es de TBD Hz</t>
-  </si>
-  <si>
-    <t>La fecha de entrega Final será el TBD para la convocatoria Extraordinaria</t>
-  </si>
-  <si>
-    <t>La fecha de entrega Final será el TBD para la convocatoria Ordinaria</t>
-  </si>
-  <si>
     <t>Referencia</t>
   </si>
   <si>
@@ -321,12 +294,6 @@
     <t>InterfazHostHS</t>
   </si>
   <si>
-    <t>La interfaz del Host con el PC se realizará con la tarjeta UM232H-B (TBC). Referencia XX en la Lista de Materiales (LM)</t>
-  </si>
-  <si>
-    <t>El lenguaje de programación utilizado para el desarrollo del software encargado del procesamiento de imagen será TBD</t>
-  </si>
-  <si>
     <t>LenguajeOpenCV</t>
   </si>
   <si>
@@ -336,12 +303,6 @@
     <t>UsoOpenCV</t>
   </si>
   <si>
-    <t>La cámara será configurable a nivel TBD</t>
-  </si>
-  <si>
-    <t>Los parámetros de configuración de la cámara son: TBD</t>
-  </si>
-  <si>
     <t>ConfiguracionCamara</t>
   </si>
   <si>
@@ -351,9 +312,6 @@
     <t>BotonesGUI</t>
   </si>
   <si>
-    <t>La ventana dedicada permitirá el control/configuración de TBD</t>
-  </si>
-  <si>
     <t>Id1</t>
   </si>
   <si>
@@ -366,17 +324,92 @@
     <t>Ordenador</t>
   </si>
   <si>
-    <t>El PC encargado de ejecutar el SW tiene el SO Windows (TBD) con las siguientes capacidades mínimas: TBD</t>
-  </si>
-  <si>
-    <t>Memoria</t>
+    <t>Formato documentación</t>
+  </si>
+  <si>
+    <t>Trabajar con tecnología de Xilinx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El producto final será autocontenido, lo ideal es que sea de tipo instalador y que no requiera de instalacion librerías </t>
+  </si>
+  <si>
+    <t>El lenguaje de programación utilizado para el desarrollo del software encargado del procesamiento de imagen será C/C++ por preferencia, aunque se podrá usar el lenguaje que sea más cómodo para el programador</t>
+  </si>
+  <si>
+    <t>Es posible que se requiera utilizar hilos diferentes para concurrencia de tareas a nivel de SW de PC</t>
+  </si>
+  <si>
+    <t>El software en el PC debe mostrar el flujo de vídeo en una ventana dedicada en tiempo real</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La ventana dedicada permitirá el control/habilitado del procesamiento de imagen: la detección de rostros </t>
+  </si>
+  <si>
+    <t>Sería deseable tener la información más relevante como el frame rate en la GUI</t>
+  </si>
+  <si>
+    <t>El PC encargado de ejecutar el SW tiene el SO Windows</t>
+  </si>
+  <si>
+    <t>RAM minima de 8Gb</t>
+  </si>
+  <si>
+    <t>La conexión del host con el ordenador se realiza mediante protocolo USB 2.0</t>
+  </si>
+  <si>
+    <t>USB 3.0 es mucho más complejo y no hay contladores tan faciles de encontrar</t>
+  </si>
+  <si>
+    <t>La Frecuencia mínima a la que deben llegar las imágenes (Frame rate) por la comunicación serie al PC es de 10Hz</t>
+  </si>
+  <si>
+    <t>Suele ser los fps de videoporteros</t>
+  </si>
+  <si>
+    <t>El sensor debe configurarse para capturar una resolución mínima de VGA</t>
+  </si>
+  <si>
+    <t>Como mínimo las imágenes tiene que ser en escala de grises (1 byte por pixel)</t>
+  </si>
+  <si>
+    <t>Deseable tener imágenes en color en la visualización manteniendo las prestaciones</t>
+  </si>
+  <si>
+    <t>Opcional medir el tiempo de flyback (orden desde PC hasta que le llega la imagen)</t>
+  </si>
+  <si>
+    <t>El PC será el encargado de solicitar una nueva imagen cuando sea capaz</t>
+  </si>
+  <si>
+    <t>La interfaz del Host con el PC se realizará con la tarjeta UM232H-B. Referencia XX en la Lista de Materiales (LM)</t>
+  </si>
+  <si>
+    <t>El retardo total desde la captura del frame hasta su visualización en el PC no debe superar varios ms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es deseable habilitar el canal que permita configurar la cámara. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deseable </t>
+  </si>
+  <si>
+    <t>Iluminación suficiente y distancia de unos 2m</t>
+  </si>
+  <si>
+    <t>Interfaz fifo asincrona -&gt; FT245</t>
+  </si>
+  <si>
+    <t>La fecha de entrega Final será el 30 Jun  para la convocatoria Ordinaria</t>
+  </si>
+  <si>
+    <t>La fecha de entrega Final será el 4 Sept para la convocatoria Extraordinaria</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -425,6 +458,12 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -472,7 +511,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -480,10 +519,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -534,7 +576,7 @@
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>781050</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -583,7 +625,7 @@
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>781050</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -632,7 +674,7 @@
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>781050</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -681,7 +723,7 @@
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>781050</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -730,7 +772,7 @@
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>781050</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -779,7 +821,7 @@
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>781050</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1153,12 +1195,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8"/>
     <col min="3" max="3" width="24.5703125"/>
-    <col min="4" max="4" width="129.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="144.140625" customWidth="1"/>
     <col min="5" max="5" width="10.5703125" style="4"/>
     <col min="6" max="6" width="15.5703125"/>
     <col min="7" max="7" width="13.5703125"/>
@@ -1170,20 +1212,20 @@
     <col min="13" max="1025" width="10.5703125"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C1" s="6" t="s">
+    <row r="1" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -1193,7 +1235,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1201,12 +1243,12 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E2" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>5</v>
       </c>
       <c r="F2" s="1"/>
@@ -1214,7 +1256,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -1222,12 +1264,12 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E3" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>5</v>
       </c>
       <c r="F3" s="1"/>
@@ -1235,41 +1277,41 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1">
         <v>1</v>
       </c>
-      <c r="B4" s="1">
-        <v>3</v>
-      </c>
       <c r="C4" s="1" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E4" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>5</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>2</v>
       </c>
       <c r="B5" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>5</v>
       </c>
       <c r="F5" s="1"/>
@@ -1277,20 +1319,20 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>2</v>
       </c>
-      <c r="B6" s="1">
-        <v>2</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>14</v>
+      <c r="B6" s="3">
+        <v>1</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>42</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E6" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>5</v>
       </c>
       <c r="F6" s="1"/>
@@ -1298,7 +1340,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>2</v>
       </c>
@@ -1306,12 +1348,12 @@
         <v>1</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>56</v>
+        <v>12</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="E7" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>5</v>
       </c>
       <c r="F7" s="1"/>
@@ -1319,62 +1361,68 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
+        <v>3</v>
+      </c>
+      <c r="B8" s="1">
         <v>2</v>
       </c>
-      <c r="B8" s="3">
-        <v>1</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>12</v>
+      <c r="C8" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>5</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H8" s="7" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B9" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E9" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>5</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H9" s="7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>4</v>
       </c>
       <c r="B10" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E10" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>5</v>
       </c>
       <c r="F10" s="1"/>
@@ -1382,20 +1430,20 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>4</v>
       </c>
       <c r="B11" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="D11" t="s">
+        <v>63</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>5</v>
       </c>
       <c r="F11" s="1"/>
@@ -1403,20 +1451,20 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B12" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" t="s">
-        <v>21</v>
-      </c>
-      <c r="E12" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>5</v>
       </c>
       <c r="F12" s="1"/>
@@ -1424,20 +1472,20 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B13" s="1">
         <v>1</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E13" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" t="s">
+        <v>48</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>5</v>
       </c>
       <c r="F13" s="1"/>
@@ -1445,20 +1493,20 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="5">
+    <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
         <v>6</v>
       </c>
-      <c r="B14" s="5">
-        <v>1</v>
+      <c r="B14" s="1">
+        <v>2</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="D14" t="s">
-        <v>22</v>
-      </c>
-      <c r="E14" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>5</v>
       </c>
       <c r="F14" s="1"/>
@@ -1466,20 +1514,20 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="5">
-        <v>6</v>
-      </c>
-      <c r="B15" s="5">
-        <v>2</v>
+    <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>7</v>
+      </c>
+      <c r="B15" s="1">
+        <v>1</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D15" t="s">
-        <v>52</v>
-      </c>
-      <c r="E15" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E15" s="5" t="s">
         <v>5</v>
       </c>
       <c r="F15" s="1"/>
@@ -1487,20 +1535,20 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>7</v>
       </c>
       <c r="B16" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E16" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E16" s="5" t="s">
         <v>5</v>
       </c>
       <c r="F16" s="1"/>
@@ -1510,18 +1558,18 @@
     </row>
     <row r="17" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B17" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E17" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="E17" s="5" t="s">
         <v>5</v>
       </c>
       <c r="F17" s="1"/>
@@ -1534,15 +1582,15 @@
         <v>8</v>
       </c>
       <c r="B18" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E18" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="E18" s="5" t="s">
         <v>5</v>
       </c>
       <c r="F18" s="1"/>
@@ -1552,50 +1600,42 @@
     </row>
     <row r="19" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B19" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E19" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D19" s="6"/>
+      <c r="E19" s="5" t="s">
         <v>5</v>
       </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1">
-        <v>9</v>
-      </c>
-      <c r="B20" s="1">
-        <v>1</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D20" s="1"/>
-      <c r="E20" s="6" t="s">
-        <v>5</v>
-      </c>
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E20" s="5"/>
       <c r="F20" s="1"/>
-      <c r="G20" s="1" t="s">
-        <v>10</v>
-      </c>
+      <c r="G20" s="1"/>
     </row>
     <row r="21" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="6"/>
+      <c r="D21" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E21" s="5"/>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
     </row>
@@ -1603,8 +1643,10 @@
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="6"/>
+      <c r="D22" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E22" s="5"/>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
     </row>
@@ -1612,19 +1654,47 @@
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="6"/>
+      <c r="D23" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E23" s="5"/>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
     </row>
-    <row r="24" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D24" s="7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D25" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D26" s="7" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D27" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D28" s="7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D29" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D30" s="9" t="s">
+        <v>67</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
@@ -1637,7 +1707,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations disablePrompts="1" count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F20" xr:uid="{4DDBC533-0419-46F1-B6B3-324F26BF199B}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F19" xr:uid="{4DDBC533-0419-46F1-B6B3-324F26BF199B}">
       <formula1>$A$2:$A$1048576</formula1>
     </dataValidation>
   </dataValidations>
@@ -1652,13 +1722,13 @@
           <x14:formula1>
             <xm:f>Listas!$A$2:$A$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E20</xm:sqref>
+          <xm:sqref>E2:E19</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{93332DCB-95CB-47BB-B0B8-5373262B883D}">
           <x14:formula1>
             <xm:f>Listas!$B$2:$B$3</xm:f>
           </x14:formula1>
-          <xm:sqref>G2:G20</xm:sqref>
+          <xm:sqref>G2:G19</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1718,19 +1788,19 @@
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="D2" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="E2" t="s">
         <v>0</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="G2" t="s">
         <v>1</v>
@@ -1738,10 +1808,10 @@
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="E3" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="F3" s="4">
         <v>1</v>
@@ -1749,10 +1819,10 @@
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="E4" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="F4" s="4">
         <v>1</v>
@@ -1760,7 +1830,7 @@
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="E5" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>